<commit_message>
Complete selenium main project
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestOutput.xlsx
+++ b/src/test/resources/testdata/TestOutput.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="60">
   <si>
     <t>S.No</t>
   </si>
@@ -187,6 +187,21 @@
   </si>
   <si>
     <t>Cabalo Solid Wood Dining Chair in Dark Walnut Finish - Set of 2</t>
+  </si>
+  <si>
+    <t>₹9,599</t>
+  </si>
+  <si>
+    <t>Rhodes Solid Wood Bookshelf in Teak Finish</t>
+  </si>
+  <si>
+    <t>₹9,999</t>
+  </si>
+  <si>
+    <t>Mika Leatherette Study Chair in White Colour</t>
+  </si>
+  <si>
+    <t>₹17,999</t>
   </si>
 </sst>
 </file>
@@ -559,7 +574,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C209"/>
+  <dimension ref="A1:C394"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -2543,6 +2558,1713 @@
     <row r="209">
       <c r="A209" t="s" s="0">
         <v>51</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n" s="0">
+        <v>209.0</v>
+      </c>
+      <c r="B210" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="C210" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n" s="0">
+        <v>210.0</v>
+      </c>
+      <c r="B211" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C211" t="s" s="0">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n" s="0">
+        <v>211.0</v>
+      </c>
+      <c r="B212" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="C212" t="s" s="0">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="s" s="0">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B216" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C216" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B217" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C217" t="s" s="0">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B218" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C218" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B219" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C219" t="s" s="0">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="B220" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="C220" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="B221" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C221" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="B222" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C222" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n" s="0">
+        <v>7.0</v>
+      </c>
+      <c r="B223" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C223" t="s" s="0">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="B224" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="C224" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n" s="0">
+        <v>9.0</v>
+      </c>
+      <c r="B225" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="C225" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="B226" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="C226" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n" s="0">
+        <v>11.0</v>
+      </c>
+      <c r="B227" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="C227" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n" s="0">
+        <v>12.0</v>
+      </c>
+      <c r="B228" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C228" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n" s="0">
+        <v>13.0</v>
+      </c>
+      <c r="B229" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="C229" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n" s="0">
+        <v>14.0</v>
+      </c>
+      <c r="B230" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C230" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="B231" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="C231" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n" s="0">
+        <v>16.0</v>
+      </c>
+      <c r="B232" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C232" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n" s="0">
+        <v>17.0</v>
+      </c>
+      <c r="B233" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C233" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n" s="0">
+        <v>18.0</v>
+      </c>
+      <c r="B234" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C234" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="B235" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="C235" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n" s="0">
+        <v>20.0</v>
+      </c>
+      <c r="B236" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C236" t="s" s="0">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="s" s="0">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="s" s="0">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="s" s="0">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n" s="0">
+        <v>241.0</v>
+      </c>
+      <c r="B242" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="C242" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n" s="0">
+        <v>242.0</v>
+      </c>
+      <c r="B243" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C243" t="s" s="0">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n" s="0">
+        <v>243.0</v>
+      </c>
+      <c r="B244" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="C244" t="s" s="0">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="s" s="0">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B248" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C248" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B249" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C249" t="s" s="0">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B250" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C250" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B251" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C251" t="s" s="0">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="B252" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="C252" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="B253" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C253" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="B254" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C254" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n" s="0">
+        <v>7.0</v>
+      </c>
+      <c r="B255" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C255" t="s" s="0">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="B256" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="C256" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n" s="0">
+        <v>9.0</v>
+      </c>
+      <c r="B257" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="C257" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="B258" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="C258" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n" s="0">
+        <v>11.0</v>
+      </c>
+      <c r="B259" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="C259" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n" s="0">
+        <v>12.0</v>
+      </c>
+      <c r="B260" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C260" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n" s="0">
+        <v>13.0</v>
+      </c>
+      <c r="B261" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="C261" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n" s="0">
+        <v>14.0</v>
+      </c>
+      <c r="B262" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C262" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="B263" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="C263" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n" s="0">
+        <v>16.0</v>
+      </c>
+      <c r="B264" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C264" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n" s="0">
+        <v>17.0</v>
+      </c>
+      <c r="B265" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C265" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n" s="0">
+        <v>18.0</v>
+      </c>
+      <c r="B266" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C266" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="B267" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="C267" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n" s="0">
+        <v>20.0</v>
+      </c>
+      <c r="B268" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C268" t="s" s="0">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="s" s="0">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="s" s="0">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="s" s="0">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n" s="0">
+        <v>273.0</v>
+      </c>
+      <c r="B274" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="C274" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n" s="0">
+        <v>274.0</v>
+      </c>
+      <c r="B275" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C275" t="s" s="0">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n" s="0">
+        <v>275.0</v>
+      </c>
+      <c r="B276" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="C276" t="s" s="0">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="s" s="0">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B280" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C280" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B281" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C281" t="s" s="0">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B282" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C282" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B283" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C283" t="s" s="0">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="B284" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="C284" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="B285" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C285" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="B286" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C286" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n" s="0">
+        <v>7.0</v>
+      </c>
+      <c r="B287" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C287" t="s" s="0">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="B288" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="C288" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="n" s="0">
+        <v>9.0</v>
+      </c>
+      <c r="B289" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="C289" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="B290" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="C290" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n" s="0">
+        <v>11.0</v>
+      </c>
+      <c r="B291" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="C291" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="n" s="0">
+        <v>12.0</v>
+      </c>
+      <c r="B292" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C292" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n" s="0">
+        <v>13.0</v>
+      </c>
+      <c r="B293" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="C293" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n" s="0">
+        <v>14.0</v>
+      </c>
+      <c r="B294" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C294" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="B295" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="C295" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n" s="0">
+        <v>16.0</v>
+      </c>
+      <c r="B296" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C296" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="n" s="0">
+        <v>17.0</v>
+      </c>
+      <c r="B297" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C297" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="n" s="0">
+        <v>18.0</v>
+      </c>
+      <c r="B298" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C298" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="n" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="B299" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="C299" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="n" s="0">
+        <v>20.0</v>
+      </c>
+      <c r="B300" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C300" t="s" s="0">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="s" s="0">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="s" s="0">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="s" s="0">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="n" s="0">
+        <v>305.0</v>
+      </c>
+      <c r="B306" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="C306" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="n" s="0">
+        <v>306.0</v>
+      </c>
+      <c r="B307" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C307" t="s" s="0">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="n" s="0">
+        <v>307.0</v>
+      </c>
+      <c r="B308" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="C308" t="s" s="0">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="s" s="0">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B312" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C312" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B313" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C313" t="s" s="0">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B314" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C314" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B315" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C315" t="s" s="0">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="B316" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="C316" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="B317" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C317" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="B318" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C318" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="n" s="0">
+        <v>7.0</v>
+      </c>
+      <c r="B319" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C319" t="s" s="0">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="B320" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="C320" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="n" s="0">
+        <v>9.0</v>
+      </c>
+      <c r="B321" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="C321" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="B322" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="C322" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="n" s="0">
+        <v>11.0</v>
+      </c>
+      <c r="B323" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="C323" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="n" s="0">
+        <v>12.0</v>
+      </c>
+      <c r="B324" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C324" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="n" s="0">
+        <v>13.0</v>
+      </c>
+      <c r="B325" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="C325" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="n" s="0">
+        <v>14.0</v>
+      </c>
+      <c r="B326" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C326" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="B327" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="C327" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="n" s="0">
+        <v>16.0</v>
+      </c>
+      <c r="B328" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C328" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="n" s="0">
+        <v>17.0</v>
+      </c>
+      <c r="B329" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C329" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="n" s="0">
+        <v>18.0</v>
+      </c>
+      <c r="B330" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C330" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="n" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="B331" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="C331" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="n" s="0">
+        <v>20.0</v>
+      </c>
+      <c r="B332" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C332" t="s" s="0">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="s" s="0">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="s" s="0">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="s" s="0">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="n" s="0">
+        <v>337.0</v>
+      </c>
+      <c r="B338" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C338" t="s" s="0">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="n" s="0">
+        <v>338.0</v>
+      </c>
+      <c r="B339" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="C339" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="n" s="0">
+        <v>339.0</v>
+      </c>
+      <c r="B340" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C340" t="s" s="0">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="n" s="0">
+        <v>340.0</v>
+      </c>
+      <c r="B341" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C341" t="s" s="0">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="n" s="0">
+        <v>341.0</v>
+      </c>
+      <c r="B342" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="C342" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="n" s="0">
+        <v>342.0</v>
+      </c>
+      <c r="B343" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C343" t="s" s="0">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="s" s="0">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B347" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C347" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B348" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C348" t="s" s="0">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B349" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C349" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B350" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C350" t="s" s="0">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="B351" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="C351" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="B352" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C352" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="B353" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C353" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="n" s="0">
+        <v>7.0</v>
+      </c>
+      <c r="B354" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C354" t="s" s="0">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="B355" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="C355" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="n" s="0">
+        <v>9.0</v>
+      </c>
+      <c r="B356" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="C356" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="B357" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="C357" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="n" s="0">
+        <v>11.0</v>
+      </c>
+      <c r="B358" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C358" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="n" s="0">
+        <v>12.0</v>
+      </c>
+      <c r="B359" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="C359" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="n" s="0">
+        <v>13.0</v>
+      </c>
+      <c r="B360" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C360" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="n" s="0">
+        <v>14.0</v>
+      </c>
+      <c r="B361" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="C361" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="B362" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C362" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="n" s="0">
+        <v>16.0</v>
+      </c>
+      <c r="B363" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C363" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="n" s="0">
+        <v>17.0</v>
+      </c>
+      <c r="B364" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C364" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="n" s="0">
+        <v>18.0</v>
+      </c>
+      <c r="B365" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="C365" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="n" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="B366" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C366" t="s" s="0">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="n" s="0">
+        <v>20.0</v>
+      </c>
+      <c r="B367" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="C367" t="s" s="0">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="n" s="0">
+        <v>367.0</v>
+      </c>
+      <c r="B368" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="C368" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="n" s="0">
+        <v>368.0</v>
+      </c>
+      <c r="B369" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C369" t="s" s="0">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="n" s="0">
+        <v>369.0</v>
+      </c>
+      <c r="B370" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="C370" t="s" s="0">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="s" s="0">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B374" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C374" t="s" s="0">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B375" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C375" t="s" s="0">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B376" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C376" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B377" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C377" t="s" s="0">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="B378" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="C378" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="B379" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C379" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="B380" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C380" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="n" s="0">
+        <v>7.0</v>
+      </c>
+      <c r="B381" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C381" t="s" s="0">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="B382" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="C382" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="n" s="0">
+        <v>9.0</v>
+      </c>
+      <c r="B383" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="C383" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="B384" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="C384" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="n" s="0">
+        <v>11.0</v>
+      </c>
+      <c r="B385" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C385" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="n" s="0">
+        <v>12.0</v>
+      </c>
+      <c r="B386" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="C386" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="n" s="0">
+        <v>13.0</v>
+      </c>
+      <c r="B387" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C387" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="n" s="0">
+        <v>14.0</v>
+      </c>
+      <c r="B388" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="C388" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="B389" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C389" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="n" s="0">
+        <v>16.0</v>
+      </c>
+      <c r="B390" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C390" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="n" s="0">
+        <v>17.0</v>
+      </c>
+      <c r="B391" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C391" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="n" s="0">
+        <v>18.0</v>
+      </c>
+      <c r="B392" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="C392" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="n" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="B393" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C393" t="s" s="0">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="n" s="0">
+        <v>20.0</v>
+      </c>
+      <c r="B394" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="C394" t="s" s="0">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -2552,7 +4274,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4018DD7B-01A5-4810-8DB3-FB76076E4E02}">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="19.0"/>
@@ -2798,6 +4520,246 @@
         <v>14</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B34" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B35" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B36" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B37" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B40" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B41" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B42" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B43" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B44" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B45" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B46" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B47" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B48" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B49" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B50" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B51" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B52" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B53" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B54" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B55" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B56" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B57" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B58" t="s" s="0">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B59" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B60" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2805,7 +4767,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -2880,6 +4842,150 @@
         <v>54</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>58</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>